<commit_message>
Update EDB source workbooks for Pages regeneration
</commit_message>
<xml_diff>
--- a/edb_data/A股-总表.xlsx
+++ b/edb_data/A股-总表.xlsx
@@ -9,7 +9,7 @@
     </mc:Choice>
   </mc:AlternateContent>
   <bookViews>
-    <workbookView windowWidth="27948" windowHeight="12300" firstSheet="1"/>
+    <workbookView windowWidth="22188" windowHeight="9060" firstSheet="1"/>
   </bookViews>
   <sheets>
     <sheet name="期权实时成本" sheetId="1" r:id="rId1"/>
@@ -1210,48 +1210,55 @@
   <volType type="realTimeData">
     <main first="WDF.RTQ">
       <tp t="n">
-        <v>6734.55</v>
+        <v>113.6</v>
         <stp/>
-        <stp>000852.SH</stp>
+        <stp>MO2612-P-6000</stp>
         <stp>LastPrice</stp>
-        <tr r="E4" s="1"/>
-        <tr r="F4" s="1"/>
-        <tr r="C4" s="1"/>
-        <tr r="D4" s="1"/>
+        <tr r="D10" s="1"/>
       </tp>
     </main>
     <main first="WDF.RTQ">
       <tp t="n">
-        <v>88</v>
+        <v>6630.78</v>
         <stp/>
-        <stp>MO2612-P-6000</stp>
+        <stp>000852.SH</stp>
         <stp>LastPrice</stp>
-        <tr r="D10" s="1"/>
+        <tr r="F4" s="1"/>
+        <tr r="C4" s="1"/>
+        <tr r="D4" s="1"/>
+        <tr r="E4" s="1"/>
+      </tp>
+    </main>
+    <main first="WDF.RTQ">
+      <tp t="s">
+        <v>#N/A</v>
+        <stp/>
+        <stp>MO2612-P-5800</stp>
+        <stp>LastPrice</stp>
         <tr r="E10" s="1"/>
       </tp>
     </main>
     <main first="WDF.RTQ">
       <tp t="n">
-        <v>-0.254</v>
+        <v>6555.8</v>
         <stp/>
-        <stp>MO2612-P-6200</stp>
-        <stp>Delta</stp>
-        <tr r="C13" s="1"/>
+        <stp>IM2612.CFE</stp>
+        <stp>LastPrice</stp>
+        <tr r="F10" s="1"/>
       </tp>
     </main>
     <main first="WDF.RTQ">
-      <tp t="n">
-        <v>-0.183</v>
+      <tp t="s">
+        <v>#N/A</v>
         <stp/>
-        <stp>MO2612-P-6000</stp>
+        <stp>MO2612-P-5800</stp>
         <stp>Delta</stp>
-        <tr r="D13" s="1"/>
         <tr r="E13" s="1"/>
       </tp>
     </main>
     <main first="WDF.RTQ">
       <tp t="n">
-        <v>129.6</v>
+        <v>165</v>
         <stp/>
         <stp>MO2612-P-6200</stp>
         <stp>LastPrice</stp>
@@ -1260,11 +1267,20 @@
     </main>
     <main first="WDF.RTQ">
       <tp t="n">
-        <v>6660</v>
+        <v>-0.2231</v>
         <stp/>
-        <stp>IM2612.CFE</stp>
-        <stp>LastPrice</stp>
-        <tr r="F10" s="1"/>
+        <stp>MO2612-P-6000</stp>
+        <stp>Delta</stp>
+        <tr r="D13" s="1"/>
+      </tp>
+    </main>
+    <main first="WDF.RTQ">
+      <tp t="n">
+        <v>-0.3028</v>
+        <stp/>
+        <stp>MO2612-P-6200</stp>
+        <stp>Delta</stp>
+        <tr r="C13" s="1"/>
       </tp>
     </main>
   </volType>
@@ -1583,19 +1599,19 @@
       </c>
       <c r="C3" s="17">
         <f ca="1" t="shared" ref="C3:F3" si="0">TODAY()</f>
-        <v>46318</v>
+        <v>46321</v>
       </c>
       <c r="D3" s="17">
         <f ca="1" t="shared" si="0"/>
-        <v>46318</v>
+        <v>46321</v>
       </c>
       <c r="E3" s="17">
         <f ca="1" t="shared" si="0"/>
-        <v>46318</v>
+        <v>46321</v>
       </c>
       <c r="F3" s="17">
         <f ca="1" t="shared" si="0"/>
-        <v>46318</v>
+        <v>46321</v>
       </c>
       <c r="H3" s="16"/>
       <c r="I3" s="16"/>
@@ -1611,19 +1627,19 @@
       </c>
       <c r="C4" s="18">
         <f t="shared" ref="C4:F4" si="1">RTD("WDF.RTQ",,"000852.SH","LastPrice")</f>
-        <v>6734.55</v>
+        <v>6630.78</v>
       </c>
       <c r="D4" s="14">
         <f t="shared" si="1"/>
-        <v>6734.55</v>
+        <v>6630.78</v>
       </c>
       <c r="E4" s="18">
         <f t="shared" si="1"/>
-        <v>6734.55</v>
+        <v>6630.78</v>
       </c>
       <c r="F4" s="14">
         <f t="shared" si="1"/>
-        <v>6734.55</v>
+        <v>6630.78</v>
       </c>
       <c r="H4" s="16"/>
       <c r="I4" s="16"/>
@@ -1647,7 +1663,7 @@
       </c>
       <c r="E5" s="14">
         <f>MAX(IF(E4*0.89&lt;=5000,FLOOR(E4*0.89,100),FLOOR(E4*0.89,200)),IF(E4&lt;=5000,MROUND(E4,100)-400,MROUND(E4,200)-800))</f>
-        <v>6000</v>
+        <v>5800</v>
       </c>
       <c r="F5" s="14" t="s">
         <v>8</v>
@@ -1674,7 +1690,7 @@
       </c>
       <c r="E6" s="14" t="str">
         <f ca="1">"MO"&amp;TEXT(DATE(YEAR(E3)+IF(MONTH(E3)&gt;=11,1,0),CHOOSE(MONTH(E3),3,6,6,6,9,9,9,12,12,12,3,3),1),"yymm")&amp;"-P-"&amp;E5</f>
-        <v>MO2612-P-6000</v>
+        <v>MO2612-P-5800</v>
       </c>
       <c r="F6" s="14" t="str">
         <f ca="1">"IM"&amp;TEXT(DATE(YEAR(F3)+IF(MONTH(F3)&gt;=11,1,0),CHOOSE(MONTH(F3),3,6,6,6,9,9,9,12,12,12,3,3),1),"yymm")&amp;".CFE"</f>
@@ -1694,15 +1710,15 @@
       </c>
       <c r="C7" s="19">
         <f>(C5-C4)/C4</f>
-        <v>-0.0793742714806483</v>
+        <v>-0.06496671583132</v>
       </c>
       <c r="D7" s="19">
         <f>(D5-D4)/D4</f>
-        <v>-0.109071875626434</v>
+        <v>-0.0951290798367612</v>
       </c>
       <c r="E7" s="19">
         <f>(E5-E4)/E4</f>
-        <v>-0.109071875626434</v>
+        <v>-0.125291443842203</v>
       </c>
       <c r="F7" s="19"/>
       <c r="H7" s="16"/>
@@ -1725,9 +1741,9 @@
         <f ca="1">[1]!w_info_lasttradingdate(D6)</f>
         <v>2026-12-18</v>
       </c>
-      <c r="E8" s="14" t="str">
+      <c r="E8" s="14">
         <f ca="1">[1]!w_info_lasttradingdate(E6)</f>
-        <v>2026-12-18</v>
+        <v>0</v>
       </c>
       <c r="F8" s="14" t="str">
         <f ca="1">[1]!s_info_ltdate_new(F6,F3)</f>
@@ -1747,19 +1763,19 @@
       </c>
       <c r="C9" s="14">
         <f ca="1" t="shared" ref="C9:F9" si="2">C8-C3</f>
-        <v>56</v>
+        <v>53</v>
       </c>
       <c r="D9" s="14">
         <f ca="1" t="shared" si="2"/>
-        <v>56</v>
+        <v>53</v>
       </c>
       <c r="E9" s="14">
         <f ca="1" t="shared" si="2"/>
-        <v>56</v>
+        <v>-46321</v>
       </c>
       <c r="F9" s="14">
         <f ca="1" t="shared" si="2"/>
-        <v>56</v>
+        <v>53</v>
       </c>
       <c r="H9" s="16"/>
       <c r="I9" s="16"/>
@@ -1775,19 +1791,19 @@
       </c>
       <c r="C10" s="20">
         <f ca="1" t="shared" ref="C10:F10" si="3">RTD("WDF.RTQ",,C6,"LastPrice")</f>
-        <v>129.6</v>
+        <v>165</v>
       </c>
       <c r="D10" s="20">
         <f ca="1" t="shared" si="3"/>
-        <v>88</v>
-      </c>
-      <c r="E10" s="20">
+        <v>113.6</v>
+      </c>
+      <c r="E10" s="20" t="str">
         <f ca="1" t="shared" si="3"/>
-        <v>88</v>
+        <v>#N/A</v>
       </c>
       <c r="F10" s="20">
         <f ca="1" t="shared" si="3"/>
-        <v>6660</v>
+        <v>6555.8</v>
       </c>
       <c r="H10" s="16"/>
       <c r="I10" s="16"/>
@@ -1803,19 +1819,19 @@
       </c>
       <c r="C11" s="21">
         <f ca="1">C10/C4</f>
-        <v>0.019244047486469</v>
+        <v>0.0248839503044891</v>
       </c>
       <c r="D11" s="21">
         <f ca="1">D10/D4</f>
-        <v>0.0130669458241456</v>
-      </c>
-      <c r="E11" s="21">
+        <v>0.0171322227550907</v>
+      </c>
+      <c r="E11" s="21" t="e">
         <f ca="1">E10/E4</f>
-        <v>0.0130669458241456</v>
+        <v>#VALUE!</v>
       </c>
       <c r="F11" s="21">
         <f ca="1">(F10/F4-1)*-1</f>
-        <v>0.0110697819453416</v>
+        <v>0.0113078702656398</v>
       </c>
     </row>
     <row r="12" ht="15.6" spans="2:14">
@@ -1824,19 +1840,19 @@
       </c>
       <c r="C12" s="21">
         <f ca="1" t="shared" ref="C12:F12" si="4">C11*(365/C9)</f>
-        <v>0.125429952367164</v>
+        <v>0.171370601153557</v>
       </c>
       <c r="D12" s="21">
         <f ca="1" t="shared" si="4"/>
-        <v>0.085168486175235</v>
-      </c>
-      <c r="E12" s="21">
+        <v>0.117986062369964</v>
+      </c>
+      <c r="E12" s="21" t="e">
         <f ca="1" t="shared" si="4"/>
-        <v>0.085168486175235</v>
+        <v>#VALUE!</v>
       </c>
       <c r="F12" s="21">
         <f ca="1" t="shared" si="4"/>
-        <v>0.0721512573223157</v>
+        <v>0.0778749556029913</v>
       </c>
     </row>
     <row r="13" ht="15.6" spans="2:14">
@@ -1845,15 +1861,15 @@
       </c>
       <c r="C13" s="14">
         <f ca="1">RTD("WDF.RTQ",,C6,"Delta")</f>
-        <v>-0.254</v>
+        <v>-0.3028</v>
       </c>
       <c r="D13" s="14">
         <f ca="1">RTD("WDF.RTQ",,D6,"Delta")</f>
-        <v>-0.183</v>
-      </c>
-      <c r="E13" s="14">
+        <v>-0.2231</v>
+      </c>
+      <c r="E13" s="14" t="str">
         <f ca="1">RTD("WDF.RTQ",,E6,"Delta")</f>
-        <v>-0.183</v>
+        <v>#N/A</v>
       </c>
       <c r="F13" s="14"/>
     </row>
@@ -1873,7 +1889,7 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr codeName="Sheet2"/>
-  <dimension ref="A1:B1030"/>
+  <dimension ref="A1:B1031"/>
   <sheetFormatPr defaultColWidth="8.73148148148148" defaultRowHeight="14.4" outlineLevelCol="1"/>
   <cols>
     <col min="1" max="1" width="21" customWidth="1"/>
@@ -1934,7 +1950,7 @@
         <v>44774</v>
       </c>
       <c r="B7" s="9" cm="1">
-        <f t="array" ref="B7">[1]!WSD(B3,B6:B6,B1,B2,"TradingCalendar=SSE","PriceAdj=F","rptType=1","Version=1","ShowParams=Y","cols=1;rows=1024")</f>
+        <f t="array" ref="B7">[1]!WSD(B3,B6:B6,B1,B2,"TradingCalendar=SSE","PriceAdj=F","rptType=1","Version=1","ShowParams=Y","cols=1;rows=1025")</f>
         <v>10.1791143839957</v>
       </c>
     </row>
@@ -10115,11 +10131,19 @@
       </c>
     </row>
     <row r="1030" spans="1:2">
-      <c r="A1030" s="10">
+      <c r="A1030" s="4">
         <v>46318</v>
       </c>
-      <c r="B1030" s="11">
+      <c r="B1030" s="9">
         <v>6.74957156033215</v>
+      </c>
+    </row>
+    <row r="1031" spans="1:2">
+      <c r="A1031" s="10">
+        <v>46321</v>
+      </c>
+      <c r="B1031" s="11">
+        <v>7.06698091548963</v>
       </c>
     </row>
   </sheetData>
@@ -10132,7 +10156,7 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr codeName="Sheet3"/>
-  <dimension ref="A1:E1459"/>
+  <dimension ref="A1:E1460"/>
   <sheetFormatPr defaultColWidth="8.88888888888889" defaultRowHeight="14.4" outlineLevelCol="4"/>
   <cols>
     <col min="1" max="1" width="11.8888888888889" customWidth="1"/>
@@ -31869,6 +31893,25 @@
         <v>0.549</v>
       </c>
     </row>
+    <row r="1460" spans="1:5">
+      <c r="A1460" s="2">
+        <v>46321</v>
+      </c>
+      <c r="B1460" s="3">
+        <v>40.6504531372946</v>
+      </c>
+      <c r="C1460" s="3">
+        <v>54.8253094590209</v>
+      </c>
+      <c r="D1460">
+        <f>PERCENTRANK(B708:B1460,B1460)</f>
+        <v>0.461</v>
+      </c>
+      <c r="E1460">
+        <f>PERCENTRANK(C708:C1460,C1460)</f>
+        <v>0.485</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <headerFooter/>

</xml_diff>

<commit_message>
Refresh EDB dashboard data for 2026-10-27
</commit_message>
<xml_diff>
--- a/edb_data/A股-总表.xlsx
+++ b/edb_data/A股-总表.xlsx
@@ -9,7 +9,7 @@
     </mc:Choice>
   </mc:AlternateContent>
   <bookViews>
-    <workbookView windowWidth="22188" windowHeight="9060" firstSheet="1"/>
+    <workbookView windowWidth="27948" windowHeight="12300" firstSheet="1"/>
   </bookViews>
   <sheets>
     <sheet name="期权实时成本" sheetId="1" r:id="rId1"/>
@@ -1210,37 +1210,55 @@
   <volType type="realTimeData">
     <main first="WDF.RTQ">
       <tp t="n">
-        <v>113.6</v>
+        <v>0</v>
         <stp/>
-        <stp>MO2612-P-6000</stp>
+        <stp>MO2612-P-5800</stp>
         <stp>LastPrice</stp>
         <tr r="D10" s="1"/>
       </tp>
     </main>
     <main first="WDF.RTQ">
       <tp t="n">
-        <v>6630.78</v>
+        <v>6427.17</v>
         <stp/>
         <stp>000852.SH</stp>
         <stp>LastPrice</stp>
         <tr r="F4" s="1"/>
-        <tr r="C4" s="1"/>
         <tr r="D4" s="1"/>
         <tr r="E4" s="1"/>
+        <tr r="C4" s="1"/>
       </tp>
     </main>
     <main first="WDF.RTQ">
       <tp t="s">
         <v>#N/A</v>
         <stp/>
+        <stp>MO2612-P-5600</stp>
+        <stp>Delta</stp>
+        <tr r="E13" s="1"/>
+      </tp>
+    </main>
+    <main first="WDF.RTQ">
+      <tp t="n">
+        <v>0</v>
+        <stp/>
         <stp>MO2612-P-5800</stp>
+        <stp>Delta</stp>
+        <tr r="D13" s="1"/>
+      </tp>
+    </main>
+    <main first="WDF.RTQ">
+      <tp t="s">
+        <v>#N/A</v>
+        <stp/>
+        <stp>MO2612-P-5600</stp>
         <stp>LastPrice</stp>
         <tr r="E10" s="1"/>
       </tp>
     </main>
     <main first="WDF.RTQ">
       <tp t="n">
-        <v>6555.8</v>
+        <v>6339.2</v>
         <stp/>
         <stp>IM2612.CFE</stp>
         <stp>LastPrice</stp>
@@ -1248,37 +1266,19 @@
       </tp>
     </main>
     <main first="WDF.RTQ">
-      <tp t="s">
-        <v>#N/A</v>
+      <tp t="n">
+        <v>172</v>
         <stp/>
-        <stp>MO2612-P-5800</stp>
-        <stp>Delta</stp>
-        <tr r="E13" s="1"/>
-      </tp>
-    </main>
-    <main first="WDF.RTQ">
-      <tp t="n">
-        <v>165</v>
-        <stp/>
-        <stp>MO2612-P-6200</stp>
+        <stp>MO2612-P-6000</stp>
         <stp>LastPrice</stp>
         <tr r="C10" s="1"/>
       </tp>
     </main>
     <main first="WDF.RTQ">
       <tp t="n">
-        <v>-0.2231</v>
+        <v>-0.3027</v>
         <stp/>
         <stp>MO2612-P-6000</stp>
-        <stp>Delta</stp>
-        <tr r="D13" s="1"/>
-      </tp>
-    </main>
-    <main first="WDF.RTQ">
-      <tp t="n">
-        <v>-0.3028</v>
-        <stp/>
-        <stp>MO2612-P-6200</stp>
         <stp>Delta</stp>
         <tr r="C13" s="1"/>
       </tp>
@@ -1298,7 +1298,6 @@
     <definedNames>
       <definedName name="s_info_name"/>
       <definedName name="s_info_ltdate_new"/>
-      <definedName name="w_info_lasttradingdate"/>
     </definedNames>
     <sheetDataSet>
       <sheetData sheetId="0"/>
@@ -1599,19 +1598,19 @@
       </c>
       <c r="C3" s="17">
         <f ca="1" t="shared" ref="C3:F3" si="0">TODAY()</f>
-        <v>46321</v>
+        <v>46322</v>
       </c>
       <c r="D3" s="17">
         <f ca="1" t="shared" si="0"/>
-        <v>46321</v>
+        <v>46322</v>
       </c>
       <c r="E3" s="17">
         <f ca="1" t="shared" si="0"/>
-        <v>46321</v>
+        <v>46322</v>
       </c>
       <c r="F3" s="17">
         <f ca="1" t="shared" si="0"/>
-        <v>46321</v>
+        <v>46322</v>
       </c>
       <c r="H3" s="16"/>
       <c r="I3" s="16"/>
@@ -1627,19 +1626,19 @@
       </c>
       <c r="C4" s="18">
         <f t="shared" ref="C4:F4" si="1">RTD("WDF.RTQ",,"000852.SH","LastPrice")</f>
-        <v>6630.78</v>
+        <v>6427.17</v>
       </c>
       <c r="D4" s="14">
         <f t="shared" si="1"/>
-        <v>6630.78</v>
+        <v>6427.17</v>
       </c>
       <c r="E4" s="18">
         <f t="shared" si="1"/>
-        <v>6630.78</v>
+        <v>6427.17</v>
       </c>
       <c r="F4" s="14">
         <f t="shared" si="1"/>
-        <v>6630.78</v>
+        <v>6427.17</v>
       </c>
       <c r="H4" s="16"/>
       <c r="I4" s="16"/>
@@ -1655,15 +1654,15 @@
       </c>
       <c r="C5" s="14">
         <f>MAX(IF(C4*0.95&lt;=5000,FLOOR(C4*0.95,100),FLOOR(C4*0.95,200)),IF(C4&lt;=5000,MROUND(C4,100)-400,MROUND(C4,200)-800))</f>
-        <v>6200</v>
+        <v>6000</v>
       </c>
       <c r="D5" s="14">
         <f>MAX(IF(D4*0.92&lt;=5000,FLOOR(D4*0.92,100),FLOOR(D4*0.92,200)),IF(D4&lt;=5000,MROUND(D4,100)-400,MROUND(D4,200)-800))</f>
-        <v>6000</v>
+        <v>5800</v>
       </c>
       <c r="E5" s="14">
         <f>MAX(IF(E4*0.89&lt;=5000,FLOOR(E4*0.89,100),FLOOR(E4*0.89,200)),IF(E4&lt;=5000,MROUND(E4,100)-400,MROUND(E4,200)-800))</f>
-        <v>5800</v>
+        <v>5600</v>
       </c>
       <c r="F5" s="14" t="s">
         <v>8</v>
@@ -1682,15 +1681,15 @@
       </c>
       <c r="C6" s="14" t="str">
         <f ca="1">"MO"&amp;TEXT(DATE(YEAR(C3)+IF(MONTH(C3)&gt;=11,1,0),CHOOSE(MONTH(C3),3,6,6,6,9,9,9,12,12,12,3,3),1),"yymm")&amp;"-P-"&amp;C5</f>
-        <v>MO2612-P-6200</v>
+        <v>MO2612-P-6000</v>
       </c>
       <c r="D6" s="14" t="str">
         <f ca="1">"MO"&amp;TEXT(DATE(YEAR(D3)+IF(MONTH(D3)&gt;=11,1,0),CHOOSE(MONTH(D3),3,6,6,6,9,9,9,12,12,12,3,3),1),"yymm")&amp;"-P-"&amp;D5</f>
-        <v>MO2612-P-6000</v>
+        <v>MO2612-P-5800</v>
       </c>
       <c r="E6" s="14" t="str">
         <f ca="1">"MO"&amp;TEXT(DATE(YEAR(E3)+IF(MONTH(E3)&gt;=11,1,0),CHOOSE(MONTH(E3),3,6,6,6,9,9,9,12,12,12,3,3),1),"yymm")&amp;"-P-"&amp;E5</f>
-        <v>MO2612-P-5800</v>
+        <v>MO2612-P-5600</v>
       </c>
       <c r="F6" s="14" t="str">
         <f ca="1">"IM"&amp;TEXT(DATE(YEAR(F3)+IF(MONTH(F3)&gt;=11,1,0),CHOOSE(MONTH(F3),3,6,6,6,9,9,9,12,12,12,3,3),1),"yymm")&amp;".CFE"</f>
@@ -1710,15 +1709,15 @@
       </c>
       <c r="C7" s="19">
         <f>(C5-C4)/C4</f>
-        <v>-0.06496671583132</v>
+        <v>-0.066463155634595</v>
       </c>
       <c r="D7" s="19">
         <f>(D5-D4)/D4</f>
-        <v>-0.0951290798367612</v>
+        <v>-0.0975810504467752</v>
       </c>
       <c r="E7" s="19">
         <f>(E5-E4)/E4</f>
-        <v>-0.125291443842203</v>
+        <v>-0.128698945258955</v>
       </c>
       <c r="F7" s="19"/>
       <c r="H7" s="16"/>
@@ -1763,19 +1762,19 @@
       </c>
       <c r="C9" s="14">
         <f ca="1" t="shared" ref="C9:F9" si="2">C8-C3</f>
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="D9" s="14">
         <f ca="1" t="shared" si="2"/>
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="E9" s="14">
         <f ca="1" t="shared" si="2"/>
-        <v>-46321</v>
+        <v>-46322</v>
       </c>
       <c r="F9" s="14">
         <f ca="1" t="shared" si="2"/>
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="H9" s="16"/>
       <c r="I9" s="16"/>
@@ -1791,11 +1790,11 @@
       </c>
       <c r="C10" s="20">
         <f ca="1" t="shared" ref="C10:F10" si="3">RTD("WDF.RTQ",,C6,"LastPrice")</f>
-        <v>165</v>
+        <v>172</v>
       </c>
       <c r="D10" s="20">
         <f ca="1" t="shared" si="3"/>
-        <v>113.6</v>
+        <v>0</v>
       </c>
       <c r="E10" s="20" t="str">
         <f ca="1" t="shared" si="3"/>
@@ -1803,7 +1802,7 @@
       </c>
       <c r="F10" s="20">
         <f ca="1" t="shared" si="3"/>
-        <v>6555.8</v>
+        <v>6339.2</v>
       </c>
       <c r="H10" s="16"/>
       <c r="I10" s="16"/>
@@ -1819,11 +1818,11 @@
       </c>
       <c r="C11" s="21">
         <f ca="1">C10/C4</f>
-        <v>0.0248839503044891</v>
+        <v>0.0267613895384749</v>
       </c>
       <c r="D11" s="21">
         <f ca="1">D10/D4</f>
-        <v>0.0171322227550907</v>
+        <v>0</v>
       </c>
       <c r="E11" s="21" t="e">
         <f ca="1">E10/E4</f>
@@ -1831,7 +1830,7 @@
       </c>
       <c r="F11" s="21">
         <f ca="1">(F10/F4-1)*-1</f>
-        <v>0.0113078702656398</v>
+        <v>0.0136872060331374</v>
       </c>
     </row>
     <row r="12" ht="15.6" spans="2:14">
@@ -1840,11 +1839,11 @@
       </c>
       <c r="C12" s="21">
         <f ca="1" t="shared" ref="C12:F12" si="4">C11*(365/C9)</f>
-        <v>0.171370601153557</v>
+        <v>0.187844368875834</v>
       </c>
       <c r="D12" s="21">
         <f ca="1" t="shared" si="4"/>
-        <v>0.117986062369964</v>
+        <v>0</v>
       </c>
       <c r="E12" s="21" t="e">
         <f ca="1" t="shared" si="4"/>
@@ -1852,7 +1851,7 @@
       </c>
       <c r="F12" s="21">
         <f ca="1" t="shared" si="4"/>
-        <v>0.0778749556029913</v>
+        <v>0.0960736577325994</v>
       </c>
     </row>
     <row r="13" ht="15.6" spans="2:14">
@@ -1861,11 +1860,11 @@
       </c>
       <c r="C13" s="14">
         <f ca="1">RTD("WDF.RTQ",,C6,"Delta")</f>
-        <v>-0.3028</v>
+        <v>-0.3027</v>
       </c>
       <c r="D13" s="14">
         <f ca="1">RTD("WDF.RTQ",,D6,"Delta")</f>
-        <v>-0.2231</v>
+        <v>0</v>
       </c>
       <c r="E13" s="14" t="str">
         <f ca="1">RTD("WDF.RTQ",,E6,"Delta")</f>
@@ -1889,7 +1888,7 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr codeName="Sheet2"/>
-  <dimension ref="A1:B1031"/>
+  <dimension ref="A1:B1032"/>
   <sheetFormatPr defaultColWidth="8.73148148148148" defaultRowHeight="14.4" outlineLevelCol="1"/>
   <cols>
     <col min="1" max="1" width="21" customWidth="1"/>
@@ -1950,7 +1949,7 @@
         <v>44774</v>
       </c>
       <c r="B7" s="9" cm="1">
-        <f t="array" ref="B7">[1]!WSD(B3,B6:B6,B1,B2,"TradingCalendar=SSE","PriceAdj=F","rptType=1","Version=1","ShowParams=Y","cols=1;rows=1025")</f>
+        <f t="array" ref="B7">[1]!WSD(B3,B6:B6,B1,B2,"TradingCalendar=SSE","PriceAdj=F","rptType=1","Version=1","ShowParams=Y","cols=1;rows=1026")</f>
         <v>10.1791143839957</v>
       </c>
     </row>
@@ -10139,11 +10138,19 @@
       </c>
     </row>
     <row r="1031" spans="1:2">
-      <c r="A1031" s="10">
+      <c r="A1031" s="4">
         <v>46321</v>
       </c>
-      <c r="B1031" s="11">
+      <c r="B1031" s="9">
         <v>7.06698091548963</v>
+      </c>
+    </row>
+    <row r="1032" spans="1:2">
+      <c r="A1032" s="10">
+        <v>46322</v>
+      </c>
+      <c r="B1032" s="11">
+        <v>8.77416481060089</v>
       </c>
     </row>
   </sheetData>
@@ -10156,7 +10163,7 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr codeName="Sheet3"/>
-  <dimension ref="A1:E1460"/>
+  <dimension ref="A1:E1461"/>
   <sheetFormatPr defaultColWidth="8.88888888888889" defaultRowHeight="14.4" outlineLevelCol="4"/>
   <cols>
     <col min="1" max="1" width="11.8888888888889" customWidth="1"/>
@@ -31912,6 +31919,25 @@
         <v>0.485</v>
       </c>
     </row>
+    <row r="1461" spans="1:5">
+      <c r="A1461" s="2">
+        <v>46322</v>
+      </c>
+      <c r="B1461" s="1">
+        <v>38.703242919937</v>
+      </c>
+      <c r="C1461" s="1">
+        <v>52.7792966772258</v>
+      </c>
+      <c r="D1461">
+        <f>PERCENTRANK(B709:B1461,B1461)</f>
+        <v>0.324</v>
+      </c>
+      <c r="E1461">
+        <f>PERCENTRANK(C709:C1461,C1461)</f>
+        <v>0.336</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <headerFooter/>

</xml_diff>

<commit_message>
Data: update EDB workbooks for 2026-10-28
</commit_message>
<xml_diff>
--- a/edb_data/A股-总表.xlsx
+++ b/edb_data/A股-总表.xlsx
@@ -9,7 +9,7 @@
     </mc:Choice>
   </mc:AlternateContent>
   <bookViews>
-    <workbookView windowWidth="27948" windowHeight="12300" firstSheet="1"/>
+    <workbookView windowWidth="22188" windowHeight="9060" firstSheet="1"/>
   </bookViews>
   <sheets>
     <sheet name="期权实时成本" sheetId="1" r:id="rId1"/>
@@ -1210,55 +1210,28 @@
   <volType type="realTimeData">
     <main first="WDF.RTQ">
       <tp t="n">
-        <v>0</v>
+        <v>122.6</v>
         <stp/>
-        <stp>MO2612-P-5800</stp>
+        <stp>MO2612-P-6000</stp>
         <stp>LastPrice</stp>
         <tr r="D10" s="1"/>
       </tp>
     </main>
     <main first="WDF.RTQ">
       <tp t="n">
-        <v>6427.17</v>
+        <v>6578.1</v>
         <stp/>
         <stp>000852.SH</stp>
         <stp>LastPrice</stp>
         <tr r="F4" s="1"/>
         <tr r="D4" s="1"/>
+        <tr r="C4" s="1"/>
         <tr r="E4" s="1"/>
-        <tr r="C4" s="1"/>
-      </tp>
-    </main>
-    <main first="WDF.RTQ">
-      <tp t="s">
-        <v>#N/A</v>
-        <stp/>
-        <stp>MO2612-P-5600</stp>
-        <stp>Delta</stp>
-        <tr r="E13" s="1"/>
       </tp>
     </main>
     <main first="WDF.RTQ">
       <tp t="n">
-        <v>0</v>
-        <stp/>
-        <stp>MO2612-P-5800</stp>
-        <stp>Delta</stp>
-        <tr r="D13" s="1"/>
-      </tp>
-    </main>
-    <main first="WDF.RTQ">
-      <tp t="s">
-        <v>#N/A</v>
-        <stp/>
-        <stp>MO2612-P-5600</stp>
-        <stp>LastPrice</stp>
-        <tr r="E10" s="1"/>
-      </tp>
-    </main>
-    <main first="WDF.RTQ">
-      <tp t="n">
-        <v>6339.2</v>
+        <v>6502</v>
         <stp/>
         <stp>IM2612.CFE</stp>
         <stp>LastPrice</stp>
@@ -1267,20 +1240,47 @@
     </main>
     <main first="WDF.RTQ">
       <tp t="n">
-        <v>172</v>
+        <v>-0.3228</v>
         <stp/>
-        <stp>MO2612-P-6000</stp>
+        <stp>MO2612-P-6200</stp>
+        <stp>Delta</stp>
+        <tr r="C13" s="1"/>
+      </tp>
+    </main>
+    <main first="WDF.RTQ">
+      <tp t="n">
+        <v>179</v>
+        <stp/>
+        <stp>MO2612-P-6200</stp>
         <stp>LastPrice</stp>
         <tr r="C10" s="1"/>
       </tp>
     </main>
     <main first="WDF.RTQ">
       <tp t="n">
-        <v>-0.3027</v>
+        <v>-0.1702</v>
+        <stp/>
+        <stp>MO2612-P-5800</stp>
+        <stp>Delta</stp>
+        <tr r="E13" s="1"/>
+      </tp>
+    </main>
+    <main first="WDF.RTQ">
+      <tp t="n">
+        <v>81.6</v>
+        <stp/>
+        <stp>MO2612-P-5800</stp>
+        <stp>LastPrice</stp>
+        <tr r="E10" s="1"/>
+      </tp>
+    </main>
+    <main first="WDF.RTQ">
+      <tp t="n">
+        <v>-0.2387</v>
         <stp/>
         <stp>MO2612-P-6000</stp>
         <stp>Delta</stp>
-        <tr r="C13" s="1"/>
+        <tr r="D13" s="1"/>
       </tp>
     </main>
   </volType>
@@ -1298,6 +1298,7 @@
     <definedNames>
       <definedName name="s_info_name"/>
       <definedName name="s_info_ltdate_new"/>
+      <definedName name="w_info_lasttradingdate"/>
     </definedNames>
     <sheetDataSet>
       <sheetData sheetId="0"/>
@@ -1598,19 +1599,19 @@
       </c>
       <c r="C3" s="17">
         <f ca="1" t="shared" ref="C3:F3" si="0">TODAY()</f>
-        <v>46322</v>
+        <v>46323</v>
       </c>
       <c r="D3" s="17">
         <f ca="1" t="shared" si="0"/>
-        <v>46322</v>
+        <v>46323</v>
       </c>
       <c r="E3" s="17">
         <f ca="1" t="shared" si="0"/>
-        <v>46322</v>
+        <v>46323</v>
       </c>
       <c r="F3" s="17">
         <f ca="1" t="shared" si="0"/>
-        <v>46322</v>
+        <v>46323</v>
       </c>
       <c r="H3" s="16"/>
       <c r="I3" s="16"/>
@@ -1626,19 +1627,19 @@
       </c>
       <c r="C4" s="18">
         <f t="shared" ref="C4:F4" si="1">RTD("WDF.RTQ",,"000852.SH","LastPrice")</f>
-        <v>6427.17</v>
+        <v>6578.1</v>
       </c>
       <c r="D4" s="14">
         <f t="shared" si="1"/>
-        <v>6427.17</v>
+        <v>6578.1</v>
       </c>
       <c r="E4" s="18">
         <f t="shared" si="1"/>
-        <v>6427.17</v>
+        <v>6578.1</v>
       </c>
       <c r="F4" s="14">
         <f t="shared" si="1"/>
-        <v>6427.17</v>
+        <v>6578.1</v>
       </c>
       <c r="H4" s="16"/>
       <c r="I4" s="16"/>
@@ -1654,15 +1655,15 @@
       </c>
       <c r="C5" s="14">
         <f>MAX(IF(C4*0.95&lt;=5000,FLOOR(C4*0.95,100),FLOOR(C4*0.95,200)),IF(C4&lt;=5000,MROUND(C4,100)-400,MROUND(C4,200)-800))</f>
-        <v>6000</v>
+        <v>6200</v>
       </c>
       <c r="D5" s="14">
         <f>MAX(IF(D4*0.92&lt;=5000,FLOOR(D4*0.92,100),FLOOR(D4*0.92,200)),IF(D4&lt;=5000,MROUND(D4,100)-400,MROUND(D4,200)-800))</f>
-        <v>5800</v>
+        <v>6000</v>
       </c>
       <c r="E5" s="14">
         <f>MAX(IF(E4*0.89&lt;=5000,FLOOR(E4*0.89,100),FLOOR(E4*0.89,200)),IF(E4&lt;=5000,MROUND(E4,100)-400,MROUND(E4,200)-800))</f>
-        <v>5600</v>
+        <v>5800</v>
       </c>
       <c r="F5" s="14" t="s">
         <v>8</v>
@@ -1681,15 +1682,15 @@
       </c>
       <c r="C6" s="14" t="str">
         <f ca="1">"MO"&amp;TEXT(DATE(YEAR(C3)+IF(MONTH(C3)&gt;=11,1,0),CHOOSE(MONTH(C3),3,6,6,6,9,9,9,12,12,12,3,3),1),"yymm")&amp;"-P-"&amp;C5</f>
-        <v>MO2612-P-6000</v>
+        <v>MO2612-P-6200</v>
       </c>
       <c r="D6" s="14" t="str">
         <f ca="1">"MO"&amp;TEXT(DATE(YEAR(D3)+IF(MONTH(D3)&gt;=11,1,0),CHOOSE(MONTH(D3),3,6,6,6,9,9,9,12,12,12,3,3),1),"yymm")&amp;"-P-"&amp;D5</f>
-        <v>MO2612-P-5800</v>
+        <v>MO2612-P-6000</v>
       </c>
       <c r="E6" s="14" t="str">
         <f ca="1">"MO"&amp;TEXT(DATE(YEAR(E3)+IF(MONTH(E3)&gt;=11,1,0),CHOOSE(MONTH(E3),3,6,6,6,9,9,9,12,12,12,3,3),1),"yymm")&amp;"-P-"&amp;E5</f>
-        <v>MO2612-P-5600</v>
+        <v>MO2612-P-5800</v>
       </c>
       <c r="F6" s="14" t="str">
         <f ca="1">"IM"&amp;TEXT(DATE(YEAR(F3)+IF(MONTH(F3)&gt;=11,1,0),CHOOSE(MONTH(F3),3,6,6,6,9,9,9,12,12,12,3,3),1),"yymm")&amp;".CFE"</f>
@@ -1709,15 +1710,15 @@
       </c>
       <c r="C7" s="19">
         <f>(C5-C4)/C4</f>
-        <v>-0.066463155634595</v>
+        <v>-0.0574786032440979</v>
       </c>
       <c r="D7" s="19">
         <f>(D5-D4)/D4</f>
-        <v>-0.0975810504467752</v>
+        <v>-0.0878825192684818</v>
       </c>
       <c r="E7" s="19">
         <f>(E5-E4)/E4</f>
-        <v>-0.128698945258955</v>
+        <v>-0.118286435292866</v>
       </c>
       <c r="F7" s="19"/>
       <c r="H7" s="16"/>
@@ -1740,9 +1741,9 @@
         <f ca="1">[1]!w_info_lasttradingdate(D6)</f>
         <v>2026-12-18</v>
       </c>
-      <c r="E8" s="14">
+      <c r="E8" s="14" t="str">
         <f ca="1">[1]!w_info_lasttradingdate(E6)</f>
-        <v>0</v>
+        <v>2026-12-18</v>
       </c>
       <c r="F8" s="14" t="str">
         <f ca="1">[1]!s_info_ltdate_new(F6,F3)</f>
@@ -1762,19 +1763,19 @@
       </c>
       <c r="C9" s="14">
         <f ca="1" t="shared" ref="C9:F9" si="2">C8-C3</f>
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="D9" s="14">
         <f ca="1" t="shared" si="2"/>
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="E9" s="14">
         <f ca="1" t="shared" si="2"/>
-        <v>-46322</v>
+        <v>51</v>
       </c>
       <c r="F9" s="14">
         <f ca="1" t="shared" si="2"/>
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="H9" s="16"/>
       <c r="I9" s="16"/>
@@ -1790,19 +1791,19 @@
       </c>
       <c r="C10" s="20">
         <f ca="1" t="shared" ref="C10:F10" si="3">RTD("WDF.RTQ",,C6,"LastPrice")</f>
-        <v>172</v>
+        <v>179</v>
       </c>
       <c r="D10" s="20">
         <f ca="1" t="shared" si="3"/>
-        <v>0</v>
-      </c>
-      <c r="E10" s="20" t="str">
+        <v>122.6</v>
+      </c>
+      <c r="E10" s="20">
         <f ca="1" t="shared" si="3"/>
-        <v>#N/A</v>
+        <v>81.6</v>
       </c>
       <c r="F10" s="20">
         <f ca="1" t="shared" si="3"/>
-        <v>6339.2</v>
+        <v>6502</v>
       </c>
       <c r="H10" s="16"/>
       <c r="I10" s="16"/>
@@ -1818,19 +1819,19 @@
       </c>
       <c r="C11" s="21">
         <f ca="1">C10/C4</f>
-        <v>0.0267613895384749</v>
+        <v>0.0272115048418236</v>
       </c>
       <c r="D11" s="21">
         <f ca="1">D10/D4</f>
-        <v>0</v>
-      </c>
-      <c r="E11" s="21" t="e">
+        <v>0.0186376005229474</v>
+      </c>
+      <c r="E11" s="21">
         <f ca="1">E10/E4</f>
-        <v>#VALUE!</v>
+        <v>0.0124047977379486</v>
       </c>
       <c r="F11" s="21">
         <f ca="1">(F10/F4-1)*-1</f>
-        <v>0.0136872060331374</v>
+        <v>0.0115686900472781</v>
       </c>
     </row>
     <row r="12" ht="15.6" spans="2:14">
@@ -1839,19 +1840,19 @@
       </c>
       <c r="C12" s="21">
         <f ca="1" t="shared" ref="C12:F12" si="4">C11*(365/C9)</f>
-        <v>0.187844368875834</v>
+        <v>0.194749005240502</v>
       </c>
       <c r="D12" s="21">
         <f ca="1" t="shared" si="4"/>
-        <v>0</v>
-      </c>
-      <c r="E12" s="21" t="e">
+        <v>0.133386748840702</v>
+      </c>
+      <c r="E12" s="21">
         <f ca="1" t="shared" si="4"/>
-        <v>#VALUE!</v>
+        <v>0.0887794347912011</v>
       </c>
       <c r="F12" s="21">
         <f ca="1" t="shared" si="4"/>
-        <v>0.0960736577325994</v>
+        <v>0.0827955268089512</v>
       </c>
     </row>
     <row r="13" ht="15.6" spans="2:14">
@@ -1860,15 +1861,15 @@
       </c>
       <c r="C13" s="14">
         <f ca="1">RTD("WDF.RTQ",,C6,"Delta")</f>
-        <v>-0.3027</v>
+        <v>-0.3228</v>
       </c>
       <c r="D13" s="14">
         <f ca="1">RTD("WDF.RTQ",,D6,"Delta")</f>
-        <v>0</v>
-      </c>
-      <c r="E13" s="14" t="str">
+        <v>-0.2387</v>
+      </c>
+      <c r="E13" s="14">
         <f ca="1">RTD("WDF.RTQ",,E6,"Delta")</f>
-        <v>#N/A</v>
+        <v>-0.1702</v>
       </c>
       <c r="F13" s="14"/>
     </row>
@@ -1888,7 +1889,7 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr codeName="Sheet2"/>
-  <dimension ref="A1:B1032"/>
+  <dimension ref="A1:B1033"/>
   <sheetFormatPr defaultColWidth="8.73148148148148" defaultRowHeight="14.4" outlineLevelCol="1"/>
   <cols>
     <col min="1" max="1" width="21" customWidth="1"/>
@@ -1949,7 +1950,7 @@
         <v>44774</v>
       </c>
       <c r="B7" s="9" cm="1">
-        <f t="array" ref="B7">[1]!WSD(B3,B6:B6,B1,B2,"TradingCalendar=SSE","PriceAdj=F","rptType=1","Version=1","ShowParams=Y","cols=1;rows=1026")</f>
+        <f t="array" ref="B7">[1]!WSD(B3,B6:B6,B1,B2,"TradingCalendar=SSE","PriceAdj=F","rptType=1","Version=1","ShowParams=Y","cols=1;rows=1027")</f>
         <v>10.1791143839957</v>
       </c>
     </row>
@@ -10146,11 +10147,19 @@
       </c>
     </row>
     <row r="1032" spans="1:2">
-      <c r="A1032" s="10">
+      <c r="A1032" s="4">
         <v>46322</v>
       </c>
-      <c r="B1032" s="11">
+      <c r="B1032" s="9">
         <v>8.77416481060089</v>
+      </c>
+    </row>
+    <row r="1033" spans="1:2">
+      <c r="A1033" s="10">
+        <v>46323</v>
+      </c>
+      <c r="B1033" s="11">
+        <v>7.61092098073832</v>
       </c>
     </row>
   </sheetData>
@@ -10163,7 +10172,7 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr codeName="Sheet3"/>
-  <dimension ref="A1:E1461"/>
+  <dimension ref="A1:E1462"/>
   <sheetFormatPr defaultColWidth="8.88888888888889" defaultRowHeight="14.4" outlineLevelCol="4"/>
   <cols>
     <col min="1" max="1" width="11.8888888888889" customWidth="1"/>
@@ -31938,6 +31947,25 @@
         <v>0.336</v>
       </c>
     </row>
+    <row r="1462" spans="1:5">
+      <c r="A1462" s="2">
+        <v>46323</v>
+      </c>
+      <c r="B1462" s="1">
+        <v>39.9712790556493</v>
+      </c>
+      <c r="C1462" s="1">
+        <v>53.787577974034</v>
+      </c>
+      <c r="D1462">
+        <f>PERCENTRANK(B710:B1462,B1462)</f>
+        <v>0.408</v>
+      </c>
+      <c r="E1462">
+        <f>PERCENTRANK(C710:C1462,C1462)</f>
+        <v>0.402</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <headerFooter/>

</xml_diff>

<commit_message>
Update EDB workbooks and dashboard data for October 29
</commit_message>
<xml_diff>
--- a/edb_data/A股-总表.xlsx
+++ b/edb_data/A股-总表.xlsx
@@ -9,7 +9,7 @@
     </mc:Choice>
   </mc:AlternateContent>
   <bookViews>
-    <workbookView windowWidth="22188" windowHeight="9060" firstSheet="1"/>
+    <workbookView windowWidth="27948" windowHeight="12300" firstSheet="1"/>
   </bookViews>
   <sheets>
     <sheet name="期权实时成本" sheetId="1" r:id="rId1"/>
@@ -1210,16 +1210,16 @@
   <volType type="realTimeData">
     <main first="WDF.RTQ">
       <tp t="n">
-        <v>122.6</v>
+        <v>128.4</v>
         <stp/>
-        <stp>MO2612-P-6000</stp>
+        <stp>MO2612-P-5800</stp>
         <stp>LastPrice</stp>
         <tr r="D10" s="1"/>
       </tp>
     </main>
     <main first="WDF.RTQ">
       <tp t="n">
-        <v>6578.1</v>
+        <v>6378.78</v>
         <stp/>
         <stp>000852.SH</stp>
         <stp>LastPrice</stp>
@@ -1231,7 +1231,43 @@
     </main>
     <main first="WDF.RTQ">
       <tp t="n">
-        <v>6502</v>
+        <v>-0.3182</v>
+        <stp/>
+        <stp>MO2612-P-6000</stp>
+        <stp>Delta</stp>
+        <tr r="C13" s="1"/>
+      </tp>
+    </main>
+    <main first="WDF.RTQ">
+      <tp t="s">
+        <v>#N/A</v>
+        <stp/>
+        <stp>MO2612-P-5600</stp>
+        <stp>Delta</stp>
+        <tr r="E13" s="1"/>
+      </tp>
+    </main>
+    <main first="WDF.RTQ">
+      <tp t="n">
+        <v>182.8</v>
+        <stp/>
+        <stp>MO2612-P-6000</stp>
+        <stp>LastPrice</stp>
+        <tr r="C10" s="1"/>
+      </tp>
+    </main>
+    <main first="WDF.RTQ">
+      <tp t="s">
+        <v>#N/A</v>
+        <stp/>
+        <stp>MO2612-P-5600</stp>
+        <stp>LastPrice</stp>
+        <tr r="E10" s="1"/>
+      </tp>
+    </main>
+    <main first="WDF.RTQ">
+      <tp t="n">
+        <v>6304.4</v>
         <stp/>
         <stp>IM2612.CFE</stp>
         <stp>LastPrice</stp>
@@ -1240,45 +1276,9 @@
     </main>
     <main first="WDF.RTQ">
       <tp t="n">
-        <v>-0.3228</v>
-        <stp/>
-        <stp>MO2612-P-6200</stp>
-        <stp>Delta</stp>
-        <tr r="C13" s="1"/>
-      </tp>
-    </main>
-    <main first="WDF.RTQ">
-      <tp t="n">
-        <v>179</v>
-        <stp/>
-        <stp>MO2612-P-6200</stp>
-        <stp>LastPrice</stp>
-        <tr r="C10" s="1"/>
-      </tp>
-    </main>
-    <main first="WDF.RTQ">
-      <tp t="n">
-        <v>-0.1702</v>
+        <v>-0.2385</v>
         <stp/>
         <stp>MO2612-P-5800</stp>
-        <stp>Delta</stp>
-        <tr r="E13" s="1"/>
-      </tp>
-    </main>
-    <main first="WDF.RTQ">
-      <tp t="n">
-        <v>81.6</v>
-        <stp/>
-        <stp>MO2612-P-5800</stp>
-        <stp>LastPrice</stp>
-        <tr r="E10" s="1"/>
-      </tp>
-    </main>
-    <main first="WDF.RTQ">
-      <tp t="n">
-        <v>-0.2387</v>
-        <stp/>
-        <stp>MO2612-P-6000</stp>
         <stp>Delta</stp>
         <tr r="D13" s="1"/>
       </tp>
@@ -1599,19 +1599,19 @@
       </c>
       <c r="C3" s="17">
         <f ca="1" t="shared" ref="C3:F3" si="0">TODAY()</f>
-        <v>46323</v>
+        <v>46324</v>
       </c>
       <c r="D3" s="17">
         <f ca="1" t="shared" si="0"/>
-        <v>46323</v>
+        <v>46324</v>
       </c>
       <c r="E3" s="17">
         <f ca="1" t="shared" si="0"/>
-        <v>46323</v>
+        <v>46324</v>
       </c>
       <c r="F3" s="17">
         <f ca="1" t="shared" si="0"/>
-        <v>46323</v>
+        <v>46324</v>
       </c>
       <c r="H3" s="16"/>
       <c r="I3" s="16"/>
@@ -1627,19 +1627,19 @@
       </c>
       <c r="C4" s="18">
         <f t="shared" ref="C4:F4" si="1">RTD("WDF.RTQ",,"000852.SH","LastPrice")</f>
-        <v>6578.1</v>
+        <v>6378.78</v>
       </c>
       <c r="D4" s="14">
         <f t="shared" si="1"/>
-        <v>6578.1</v>
+        <v>6378.78</v>
       </c>
       <c r="E4" s="18">
         <f t="shared" si="1"/>
-        <v>6578.1</v>
+        <v>6378.78</v>
       </c>
       <c r="F4" s="14">
         <f t="shared" si="1"/>
-        <v>6578.1</v>
+        <v>6378.78</v>
       </c>
       <c r="H4" s="16"/>
       <c r="I4" s="16"/>
@@ -1655,15 +1655,15 @@
       </c>
       <c r="C5" s="14">
         <f>MAX(IF(C4*0.95&lt;=5000,FLOOR(C4*0.95,100),FLOOR(C4*0.95,200)),IF(C4&lt;=5000,MROUND(C4,100)-400,MROUND(C4,200)-800))</f>
-        <v>6200</v>
+        <v>6000</v>
       </c>
       <c r="D5" s="14">
         <f>MAX(IF(D4*0.92&lt;=5000,FLOOR(D4*0.92,100),FLOOR(D4*0.92,200)),IF(D4&lt;=5000,MROUND(D4,100)-400,MROUND(D4,200)-800))</f>
-        <v>6000</v>
+        <v>5800</v>
       </c>
       <c r="E5" s="14">
         <f>MAX(IF(E4*0.89&lt;=5000,FLOOR(E4*0.89,100),FLOOR(E4*0.89,200)),IF(E4&lt;=5000,MROUND(E4,100)-400,MROUND(E4,200)-800))</f>
-        <v>5800</v>
+        <v>5600</v>
       </c>
       <c r="F5" s="14" t="s">
         <v>8</v>
@@ -1682,15 +1682,15 @@
       </c>
       <c r="C6" s="14" t="str">
         <f ca="1">"MO"&amp;TEXT(DATE(YEAR(C3)+IF(MONTH(C3)&gt;=11,1,0),CHOOSE(MONTH(C3),3,6,6,6,9,9,9,12,12,12,3,3),1),"yymm")&amp;"-P-"&amp;C5</f>
-        <v>MO2612-P-6200</v>
+        <v>MO2612-P-6000</v>
       </c>
       <c r="D6" s="14" t="str">
         <f ca="1">"MO"&amp;TEXT(DATE(YEAR(D3)+IF(MONTH(D3)&gt;=11,1,0),CHOOSE(MONTH(D3),3,6,6,6,9,9,9,12,12,12,3,3),1),"yymm")&amp;"-P-"&amp;D5</f>
-        <v>MO2612-P-6000</v>
+        <v>MO2612-P-5800</v>
       </c>
       <c r="E6" s="14" t="str">
         <f ca="1">"MO"&amp;TEXT(DATE(YEAR(E3)+IF(MONTH(E3)&gt;=11,1,0),CHOOSE(MONTH(E3),3,6,6,6,9,9,9,12,12,12,3,3),1),"yymm")&amp;"-P-"&amp;E5</f>
-        <v>MO2612-P-5800</v>
+        <v>MO2612-P-5600</v>
       </c>
       <c r="F6" s="14" t="str">
         <f ca="1">"IM"&amp;TEXT(DATE(YEAR(F3)+IF(MONTH(F3)&gt;=11,1,0),CHOOSE(MONTH(F3),3,6,6,6,9,9,9,12,12,12,3,3),1),"yymm")&amp;".CFE"</f>
@@ -1710,15 +1710,15 @@
       </c>
       <c r="C7" s="19">
         <f>(C5-C4)/C4</f>
-        <v>-0.0574786032440979</v>
+        <v>-0.0593812609934815</v>
       </c>
       <c r="D7" s="19">
         <f>(D5-D4)/D4</f>
-        <v>-0.0878825192684818</v>
+        <v>-0.0907352189603654</v>
       </c>
       <c r="E7" s="19">
         <f>(E5-E4)/E4</f>
-        <v>-0.118286435292866</v>
+        <v>-0.122089176927249</v>
       </c>
       <c r="F7" s="19"/>
       <c r="H7" s="16"/>
@@ -1741,9 +1741,9 @@
         <f ca="1">[1]!w_info_lasttradingdate(D6)</f>
         <v>2026-12-18</v>
       </c>
-      <c r="E8" s="14" t="str">
+      <c r="E8" s="14">
         <f ca="1">[1]!w_info_lasttradingdate(E6)</f>
-        <v>2026-12-18</v>
+        <v>0</v>
       </c>
       <c r="F8" s="14" t="str">
         <f ca="1">[1]!s_info_ltdate_new(F6,F3)</f>
@@ -1763,19 +1763,19 @@
       </c>
       <c r="C9" s="14">
         <f ca="1" t="shared" ref="C9:F9" si="2">C8-C3</f>
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="D9" s="14">
         <f ca="1" t="shared" si="2"/>
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="E9" s="14">
         <f ca="1" t="shared" si="2"/>
-        <v>51</v>
+        <v>-46324</v>
       </c>
       <c r="F9" s="14">
         <f ca="1" t="shared" si="2"/>
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="H9" s="16"/>
       <c r="I9" s="16"/>
@@ -1791,19 +1791,19 @@
       </c>
       <c r="C10" s="20">
         <f ca="1" t="shared" ref="C10:F10" si="3">RTD("WDF.RTQ",,C6,"LastPrice")</f>
-        <v>179</v>
+        <v>182.8</v>
       </c>
       <c r="D10" s="20">
         <f ca="1" t="shared" si="3"/>
-        <v>122.6</v>
-      </c>
-      <c r="E10" s="20">
+        <v>128.4</v>
+      </c>
+      <c r="E10" s="20" t="str">
         <f ca="1" t="shared" si="3"/>
-        <v>81.6</v>
+        <v>#N/A</v>
       </c>
       <c r="F10" s="20">
         <f ca="1" t="shared" si="3"/>
-        <v>6502</v>
+        <v>6304.4</v>
       </c>
       <c r="H10" s="16"/>
       <c r="I10" s="16"/>
@@ -1819,19 +1819,19 @@
       </c>
       <c r="C11" s="21">
         <f ca="1">C10/C4</f>
-        <v>0.0272115048418236</v>
+        <v>0.0286575175817319</v>
       </c>
       <c r="D11" s="21">
         <f ca="1">D10/D4</f>
-        <v>0.0186376005229474</v>
-      </c>
-      <c r="E11" s="21">
+        <v>0.0201292410147395</v>
+      </c>
+      <c r="E11" s="21" t="e">
         <f ca="1">E10/E4</f>
-        <v>0.0124047977379486</v>
+        <v>#VALUE!</v>
       </c>
       <c r="F11" s="21">
         <f ca="1">(F10/F4-1)*-1</f>
-        <v>0.0115686900472781</v>
+        <v>0.011660536967884</v>
       </c>
     </row>
     <row r="12" ht="15.6" spans="2:14">
@@ -1840,19 +1840,19 @@
       </c>
       <c r="C12" s="21">
         <f ca="1" t="shared" ref="C12:F12" si="4">C11*(365/C9)</f>
-        <v>0.194749005240502</v>
+        <v>0.209199878346643</v>
       </c>
       <c r="D12" s="21">
         <f ca="1" t="shared" si="4"/>
-        <v>0.133386748840702</v>
-      </c>
-      <c r="E12" s="21">
+        <v>0.146943459407598</v>
+      </c>
+      <c r="E12" s="21" t="e">
         <f ca="1" t="shared" si="4"/>
-        <v>0.0887794347912011</v>
+        <v>#VALUE!</v>
       </c>
       <c r="F12" s="21">
         <f ca="1" t="shared" si="4"/>
-        <v>0.0827955268089512</v>
+        <v>0.0851219198655536</v>
       </c>
     </row>
     <row r="13" ht="15.6" spans="2:14">
@@ -1861,15 +1861,15 @@
       </c>
       <c r="C13" s="14">
         <f ca="1">RTD("WDF.RTQ",,C6,"Delta")</f>
-        <v>-0.3228</v>
+        <v>-0.3182</v>
       </c>
       <c r="D13" s="14">
         <f ca="1">RTD("WDF.RTQ",,D6,"Delta")</f>
-        <v>-0.2387</v>
-      </c>
-      <c r="E13" s="14">
+        <v>-0.2385</v>
+      </c>
+      <c r="E13" s="14" t="str">
         <f ca="1">RTD("WDF.RTQ",,E6,"Delta")</f>
-        <v>-0.1702</v>
+        <v>#N/A</v>
       </c>
       <c r="F13" s="14"/>
     </row>
@@ -1889,7 +1889,7 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr codeName="Sheet2"/>
-  <dimension ref="A1:B1033"/>
+  <dimension ref="A1:B1034"/>
   <sheetFormatPr defaultColWidth="8.73148148148148" defaultRowHeight="14.4" outlineLevelCol="1"/>
   <cols>
     <col min="1" max="1" width="21" customWidth="1"/>
@@ -1950,7 +1950,7 @@
         <v>44774</v>
       </c>
       <c r="B7" s="9" cm="1">
-        <f t="array" ref="B7">[1]!WSD(B3,B6:B6,B1,B2,"TradingCalendar=SSE","PriceAdj=F","rptType=1","Version=1","ShowParams=Y","cols=1;rows=1027")</f>
+        <f t="array" ref="B7">[1]!WSD(B3,B6:B6,B1,B2,"TradingCalendar=SSE","PriceAdj=F","rptType=1","Version=1","ShowParams=Y","cols=1;rows=1028")</f>
         <v>10.1791143839957</v>
       </c>
     </row>
@@ -10155,11 +10155,19 @@
       </c>
     </row>
     <row r="1033" spans="1:2">
-      <c r="A1033" s="10">
+      <c r="A1033" s="4">
         <v>46323</v>
       </c>
-      <c r="B1033" s="11">
+      <c r="B1033" s="9">
         <v>7.61092098073832</v>
+      </c>
+    </row>
+    <row r="1034" spans="1:2">
+      <c r="A1034" s="10">
+        <v>46324</v>
+      </c>
+      <c r="B1034" s="11">
+        <v>7.87876213259272</v>
       </c>
     </row>
   </sheetData>
@@ -10172,7 +10180,7 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr codeName="Sheet3"/>
-  <dimension ref="A1:E1462"/>
+  <dimension ref="A1:E1463"/>
   <sheetFormatPr defaultColWidth="8.88888888888889" defaultRowHeight="14.4" outlineLevelCol="4"/>
   <cols>
     <col min="1" max="1" width="11.8888888888889" customWidth="1"/>
@@ -31966,6 +31974,25 @@
         <v>0.402</v>
       </c>
     </row>
+    <row r="1463" spans="1:5">
+      <c r="A1463" s="2">
+        <v>46324</v>
+      </c>
+      <c r="B1463" s="1">
+        <v>39.1536628496001</v>
+      </c>
+      <c r="C1463" s="1">
+        <v>53.3205119212353</v>
+      </c>
+      <c r="D1463">
+        <f>PERCENTRANK(B711:B1463,B1463)</f>
+        <v>0.361</v>
+      </c>
+      <c r="E1463">
+        <f>PERCENTRANK(C711:C1463,C1463)</f>
+        <v>0.363</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <headerFooter/>

</xml_diff>

<commit_message>
Update EDB workbooks and dashboard data for October 30
</commit_message>
<xml_diff>
--- a/edb_data/A股-总表.xlsx
+++ b/edb_data/A股-总表.xlsx
@@ -9,7 +9,7 @@
     </mc:Choice>
   </mc:AlternateContent>
   <bookViews>
-    <workbookView windowWidth="27948" windowHeight="12300" firstSheet="1"/>
+    <workbookView windowWidth="27948" windowHeight="12300" firstSheet="1" activeTab="2"/>
   </bookViews>
   <sheets>
     <sheet name="期权实时成本" sheetId="1" r:id="rId1"/>
@@ -1209,49 +1209,40 @@
 <volTypes xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <volType type="realTimeData">
     <main first="WDF.RTQ">
-      <tp t="n">
-        <v>128.4</v>
+      <tp t="s">
+        <v>#N/A</v>
         <stp/>
-        <stp>MO2612-P-5800</stp>
+        <stp>MO2612-P-5600</stp>
         <stp>LastPrice</stp>
         <tr r="D10" s="1"/>
       </tp>
     </main>
     <main first="WDF.RTQ">
       <tp t="n">
-        <v>6378.78</v>
+        <v>6161.23</v>
         <stp/>
         <stp>000852.SH</stp>
         <stp>LastPrice</stp>
         <tr r="F4" s="1"/>
-        <tr r="D4" s="1"/>
         <tr r="C4" s="1"/>
         <tr r="E4" s="1"/>
+        <tr r="D4" s="1"/>
       </tp>
     </main>
     <main first="WDF.RTQ">
       <tp t="n">
-        <v>-0.3182</v>
+        <v>-0.3352</v>
         <stp/>
-        <stp>MO2612-P-6000</stp>
+        <stp>MO2612-P-5800</stp>
         <stp>Delta</stp>
         <tr r="C13" s="1"/>
       </tp>
     </main>
     <main first="WDF.RTQ">
-      <tp t="s">
-        <v>#N/A</v>
+      <tp t="n">
+        <v>198.8</v>
         <stp/>
-        <stp>MO2612-P-5600</stp>
-        <stp>Delta</stp>
-        <tr r="E13" s="1"/>
-      </tp>
-    </main>
-    <main first="WDF.RTQ">
-      <tp t="n">
-        <v>182.8</v>
-        <stp/>
-        <stp>MO2612-P-6000</stp>
+        <stp>MO2612-P-5800</stp>
         <stp>LastPrice</stp>
         <tr r="C10" s="1"/>
       </tp>
@@ -1260,14 +1251,14 @@
       <tp t="s">
         <v>#N/A</v>
         <stp/>
-        <stp>MO2612-P-5600</stp>
+        <stp>MO2612-P-5400</stp>
         <stp>LastPrice</stp>
         <tr r="E10" s="1"/>
       </tp>
     </main>
     <main first="WDF.RTQ">
       <tp t="n">
-        <v>6304.4</v>
+        <v>6081</v>
         <stp/>
         <stp>IM2612.CFE</stp>
         <stp>LastPrice</stp>
@@ -1275,10 +1266,19 @@
       </tp>
     </main>
     <main first="WDF.RTQ">
-      <tp t="n">
-        <v>-0.2385</v>
+      <tp t="s">
+        <v>#N/A</v>
         <stp/>
-        <stp>MO2612-P-5800</stp>
+        <stp>MO2612-P-5400</stp>
+        <stp>Delta</stp>
+        <tr r="E13" s="1"/>
+      </tp>
+    </main>
+    <main first="WDF.RTQ">
+      <tp t="s">
+        <v>#N/A</v>
+        <stp/>
+        <stp>MO2612-P-5600</stp>
         <stp>Delta</stp>
         <tr r="D13" s="1"/>
       </tp>
@@ -1599,19 +1599,19 @@
       </c>
       <c r="C3" s="17">
         <f ca="1" t="shared" ref="C3:F3" si="0">TODAY()</f>
-        <v>46324</v>
+        <v>46325</v>
       </c>
       <c r="D3" s="17">
         <f ca="1" t="shared" si="0"/>
-        <v>46324</v>
+        <v>46325</v>
       </c>
       <c r="E3" s="17">
         <f ca="1" t="shared" si="0"/>
-        <v>46324</v>
+        <v>46325</v>
       </c>
       <c r="F3" s="17">
         <f ca="1" t="shared" si="0"/>
-        <v>46324</v>
+        <v>46325</v>
       </c>
       <c r="H3" s="16"/>
       <c r="I3" s="16"/>
@@ -1627,19 +1627,19 @@
       </c>
       <c r="C4" s="18">
         <f t="shared" ref="C4:F4" si="1">RTD("WDF.RTQ",,"000852.SH","LastPrice")</f>
-        <v>6378.78</v>
+        <v>6161.23</v>
       </c>
       <c r="D4" s="14">
         <f t="shared" si="1"/>
-        <v>6378.78</v>
+        <v>6161.23</v>
       </c>
       <c r="E4" s="18">
         <f t="shared" si="1"/>
-        <v>6378.78</v>
+        <v>6161.23</v>
       </c>
       <c r="F4" s="14">
         <f t="shared" si="1"/>
-        <v>6378.78</v>
+        <v>6161.23</v>
       </c>
       <c r="H4" s="16"/>
       <c r="I4" s="16"/>
@@ -1655,15 +1655,15 @@
       </c>
       <c r="C5" s="14">
         <f>MAX(IF(C4*0.95&lt;=5000,FLOOR(C4*0.95,100),FLOOR(C4*0.95,200)),IF(C4&lt;=5000,MROUND(C4,100)-400,MROUND(C4,200)-800))</f>
-        <v>6000</v>
+        <v>5800</v>
       </c>
       <c r="D5" s="14">
         <f>MAX(IF(D4*0.92&lt;=5000,FLOOR(D4*0.92,100),FLOOR(D4*0.92,200)),IF(D4&lt;=5000,MROUND(D4,100)-400,MROUND(D4,200)-800))</f>
-        <v>5800</v>
+        <v>5600</v>
       </c>
       <c r="E5" s="14">
         <f>MAX(IF(E4*0.89&lt;=5000,FLOOR(E4*0.89,100),FLOOR(E4*0.89,200)),IF(E4&lt;=5000,MROUND(E4,100)-400,MROUND(E4,200)-800))</f>
-        <v>5600</v>
+        <v>5400</v>
       </c>
       <c r="F5" s="14" t="s">
         <v>8</v>
@@ -1682,15 +1682,15 @@
       </c>
       <c r="C6" s="14" t="str">
         <f ca="1">"MO"&amp;TEXT(DATE(YEAR(C3)+IF(MONTH(C3)&gt;=11,1,0),CHOOSE(MONTH(C3),3,6,6,6,9,9,9,12,12,12,3,3),1),"yymm")&amp;"-P-"&amp;C5</f>
-        <v>MO2612-P-6000</v>
+        <v>MO2612-P-5800</v>
       </c>
       <c r="D6" s="14" t="str">
         <f ca="1">"MO"&amp;TEXT(DATE(YEAR(D3)+IF(MONTH(D3)&gt;=11,1,0),CHOOSE(MONTH(D3),3,6,6,6,9,9,9,12,12,12,3,3),1),"yymm")&amp;"-P-"&amp;D5</f>
-        <v>MO2612-P-5800</v>
+        <v>MO2612-P-5600</v>
       </c>
       <c r="E6" s="14" t="str">
         <f ca="1">"MO"&amp;TEXT(DATE(YEAR(E3)+IF(MONTH(E3)&gt;=11,1,0),CHOOSE(MONTH(E3),3,6,6,6,9,9,9,12,12,12,3,3),1),"yymm")&amp;"-P-"&amp;E5</f>
-        <v>MO2612-P-5600</v>
+        <v>MO2612-P-5400</v>
       </c>
       <c r="F6" s="14" t="str">
         <f ca="1">"IM"&amp;TEXT(DATE(YEAR(F3)+IF(MONTH(F3)&gt;=11,1,0),CHOOSE(MONTH(F3),3,6,6,6,9,9,9,12,12,12,3,3),1),"yymm")&amp;".CFE"</f>
@@ -1710,15 +1710,15 @@
       </c>
       <c r="C7" s="19">
         <f>(C5-C4)/C4</f>
-        <v>-0.0593812609934815</v>
+        <v>-0.0586295268964152</v>
       </c>
       <c r="D7" s="19">
         <f>(D5-D4)/D4</f>
-        <v>-0.0907352189603654</v>
+        <v>-0.0910905776930906</v>
       </c>
       <c r="E7" s="19">
         <f>(E5-E4)/E4</f>
-        <v>-0.122089176927249</v>
+        <v>-0.123551628489766</v>
       </c>
       <c r="F7" s="19"/>
       <c r="H7" s="16"/>
@@ -1737,9 +1737,9 @@
         <f ca="1">[1]!w_info_lasttradingdate(C6)</f>
         <v>2026-12-18</v>
       </c>
-      <c r="D8" s="14" t="str">
+      <c r="D8" s="14">
         <f ca="1">[1]!w_info_lasttradingdate(D6)</f>
-        <v>2026-12-18</v>
+        <v>0</v>
       </c>
       <c r="E8" s="14">
         <f ca="1">[1]!w_info_lasttradingdate(E6)</f>
@@ -1763,19 +1763,19 @@
       </c>
       <c r="C9" s="14">
         <f ca="1" t="shared" ref="C9:F9" si="2">C8-C3</f>
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="D9" s="14">
         <f ca="1" t="shared" si="2"/>
-        <v>50</v>
+        <v>-46325</v>
       </c>
       <c r="E9" s="14">
         <f ca="1" t="shared" si="2"/>
-        <v>-46324</v>
+        <v>-46325</v>
       </c>
       <c r="F9" s="14">
         <f ca="1" t="shared" si="2"/>
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="H9" s="16"/>
       <c r="I9" s="16"/>
@@ -1791,11 +1791,11 @@
       </c>
       <c r="C10" s="20">
         <f ca="1" t="shared" ref="C10:F10" si="3">RTD("WDF.RTQ",,C6,"LastPrice")</f>
-        <v>182.8</v>
-      </c>
-      <c r="D10" s="20">
+        <v>198.8</v>
+      </c>
+      <c r="D10" s="20" t="str">
         <f ca="1" t="shared" si="3"/>
-        <v>128.4</v>
+        <v>#N/A</v>
       </c>
       <c r="E10" s="20" t="str">
         <f ca="1" t="shared" si="3"/>
@@ -1803,7 +1803,7 @@
       </c>
       <c r="F10" s="20">
         <f ca="1" t="shared" si="3"/>
-        <v>6304.4</v>
+        <v>6081</v>
       </c>
       <c r="H10" s="16"/>
       <c r="I10" s="16"/>
@@ -1819,11 +1819,11 @@
       </c>
       <c r="C11" s="21">
         <f ca="1">C10/C4</f>
-        <v>0.0286575175817319</v>
-      </c>
-      <c r="D11" s="21">
+        <v>0.0322662844918953</v>
+      </c>
+      <c r="D11" s="21" t="e">
         <f ca="1">D10/D4</f>
-        <v>0.0201292410147395</v>
+        <v>#VALUE!</v>
       </c>
       <c r="E11" s="21" t="e">
         <f ca="1">E10/E4</f>
@@ -1831,7 +1831,7 @@
       </c>
       <c r="F11" s="21">
         <f ca="1">(F10/F4-1)*-1</f>
-        <v>0.011660536967884</v>
+        <v>0.0130217505270864</v>
       </c>
     </row>
     <row r="12" ht="15.6" spans="2:14">
@@ -1840,11 +1840,11 @@
       </c>
       <c r="C12" s="21">
         <f ca="1" t="shared" ref="C12:F12" si="4">C11*(365/C9)</f>
-        <v>0.209199878346643</v>
-      </c>
-      <c r="D12" s="21">
+        <v>0.240350894684526</v>
+      </c>
+      <c r="D12" s="21" t="e">
         <f ca="1" t="shared" si="4"/>
-        <v>0.146943459407598</v>
+        <v>#VALUE!</v>
       </c>
       <c r="E12" s="21" t="e">
         <f ca="1" t="shared" si="4"/>
@@ -1852,7 +1852,7 @@
       </c>
       <c r="F12" s="21">
         <f ca="1" t="shared" si="4"/>
-        <v>0.0851219198655536</v>
+        <v>0.0969987539262561</v>
       </c>
     </row>
     <row r="13" ht="15.6" spans="2:14">
@@ -1861,11 +1861,11 @@
       </c>
       <c r="C13" s="14">
         <f ca="1">RTD("WDF.RTQ",,C6,"Delta")</f>
-        <v>-0.3182</v>
-      </c>
-      <c r="D13" s="14">
+        <v>-0.3352</v>
+      </c>
+      <c r="D13" s="14" t="str">
         <f ca="1">RTD("WDF.RTQ",,D6,"Delta")</f>
-        <v>-0.2385</v>
+        <v>#N/A</v>
       </c>
       <c r="E13" s="14" t="str">
         <f ca="1">RTD("WDF.RTQ",,E6,"Delta")</f>
@@ -1889,7 +1889,7 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr codeName="Sheet2"/>
-  <dimension ref="A1:B1034"/>
+  <dimension ref="A1:B1035"/>
   <sheetFormatPr defaultColWidth="8.73148148148148" defaultRowHeight="14.4" outlineLevelCol="1"/>
   <cols>
     <col min="1" max="1" width="21" customWidth="1"/>
@@ -1950,7 +1950,7 @@
         <v>44774</v>
       </c>
       <c r="B7" s="9" cm="1">
-        <f t="array" ref="B7">[1]!WSD(B3,B6:B6,B1,B2,"TradingCalendar=SSE","PriceAdj=F","rptType=1","Version=1","ShowParams=Y","cols=1;rows=1028")</f>
+        <f t="array" ref="B7">[1]!WSD(B3,B6:B6,B1,B2,"TradingCalendar=SSE","PriceAdj=F","rptType=1","Version=1","ShowParams=Y","cols=1;rows=1029")</f>
         <v>10.1791143839957</v>
       </c>
     </row>
@@ -10163,11 +10163,19 @@
       </c>
     </row>
     <row r="1034" spans="1:2">
-      <c r="A1034" s="10">
+      <c r="A1034" s="4">
         <v>46324</v>
       </c>
-      <c r="B1034" s="11">
+      <c r="B1034" s="9">
         <v>7.87876213259272</v>
+      </c>
+    </row>
+    <row r="1035" spans="1:2">
+      <c r="A1035" s="10">
+        <v>46325</v>
+      </c>
+      <c r="B1035" s="11">
+        <v>-15.7011205438649</v>
       </c>
     </row>
   </sheetData>
@@ -10180,7 +10188,7 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr codeName="Sheet3"/>
-  <dimension ref="A1:E1463"/>
+  <dimension ref="A1:E1464"/>
   <sheetFormatPr defaultColWidth="8.88888888888889" defaultRowHeight="14.4" outlineLevelCol="4"/>
   <cols>
     <col min="1" max="1" width="11.8888888888889" customWidth="1"/>
@@ -31890,11 +31898,11 @@
         <v>58.9291298596294</v>
       </c>
       <c r="D1458">
-        <f>PERCENTRANK(B706:B1458,B1458)</f>
+        <f t="shared" ref="D1458:D1463" si="22">PERCENTRANK(B706:B1458,B1458)</f>
         <v>0.809</v>
       </c>
       <c r="E1458">
-        <f>PERCENTRANK(C706:C1458,C1458)</f>
+        <f t="shared" ref="E1458:E1463" si="23">PERCENTRANK(C706:C1458,C1458)</f>
         <v>0.813</v>
       </c>
     </row>
@@ -31909,11 +31917,11 @@
         <v>55.7804693973789</v>
       </c>
       <c r="D1459">
-        <f>PERCENTRANK(B707:B1459,B1459)</f>
+        <f t="shared" si="22"/>
         <v>0.578</v>
       </c>
       <c r="E1459">
-        <f>PERCENTRANK(C707:C1459,C1459)</f>
+        <f t="shared" si="23"/>
         <v>0.549</v>
       </c>
     </row>
@@ -31928,11 +31936,11 @@
         <v>54.8253094590209</v>
       </c>
       <c r="D1460">
-        <f>PERCENTRANK(B708:B1460,B1460)</f>
+        <f t="shared" si="22"/>
         <v>0.461</v>
       </c>
       <c r="E1460">
-        <f>PERCENTRANK(C708:C1460,C1460)</f>
+        <f t="shared" si="23"/>
         <v>0.485</v>
       </c>
     </row>
@@ -31947,11 +31955,11 @@
         <v>52.7792966772258</v>
       </c>
       <c r="D1461">
-        <f>PERCENTRANK(B709:B1461,B1461)</f>
+        <f t="shared" si="22"/>
         <v>0.324</v>
       </c>
       <c r="E1461">
-        <f>PERCENTRANK(C709:C1461,C1461)</f>
+        <f t="shared" si="23"/>
         <v>0.336</v>
       </c>
     </row>
@@ -31966,11 +31974,11 @@
         <v>53.787577974034</v>
       </c>
       <c r="D1462">
-        <f>PERCENTRANK(B710:B1462,B1462)</f>
+        <f t="shared" si="22"/>
         <v>0.408</v>
       </c>
       <c r="E1462">
-        <f>PERCENTRANK(C710:C1462,C1462)</f>
+        <f t="shared" si="23"/>
         <v>0.402</v>
       </c>
     </row>
@@ -31985,12 +31993,31 @@
         <v>53.3205119212353</v>
       </c>
       <c r="D1463">
-        <f>PERCENTRANK(B711:B1463,B1463)</f>
+        <f t="shared" si="22"/>
         <v>0.361</v>
       </c>
       <c r="E1463">
-        <f>PERCENTRANK(C711:C1463,C1463)</f>
+        <f t="shared" si="23"/>
         <v>0.363</v>
+      </c>
+    </row>
+    <row r="1464" spans="1:5">
+      <c r="A1464" s="2">
+        <v>46325</v>
+      </c>
+      <c r="B1464" s="1">
+        <v>37.5113132439701</v>
+      </c>
+      <c r="C1464" s="1">
+        <v>51.314727852582</v>
+      </c>
+      <c r="D1464">
+        <f>PERCENTRANK(B712:B1464,B1464)</f>
+        <v>0.23</v>
+      </c>
+      <c r="E1464">
+        <f>PERCENTRANK(C712:C1464,C1464)</f>
+        <v>0.22</v>
       </c>
     </row>
   </sheetData>

</xml_diff>